<commit_message>
docs(tracker): update Bug-002 status with Part Number PDF fallback elimination details
</commit_message>
<xml_diff>
--- a/tracker_updated_with_recent_commits.xlsx
+++ b/tracker_updated_with_recent_commits.xlsx
@@ -4140,7 +4140,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.63" customWidth="1" style="30" min="1" max="2"/>
@@ -4276,11 +4276,21 @@
       </c>
       <c r="G3" s="18" t="inlineStr">
         <is>
-          <t>WIll be discussing with Rajeshwari</t>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fixed in commit 5665bee: completely removed PDF filename fallbacks across extractor, spares API, and exporter, leaving part_number null when not in manual. Cleaned 3,053 legacy records.</t>
         </is>
       </c>
       <c r="J3" s="11" t="n">
         <v>46302</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Drawing No. Issue Fixed; Part No. PDF filename fallback completely eliminated (commit 5665bee)</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -4420,7 +4430,7 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="0" t="inlineStr">
         <is>
           <t>Verified on Staging: Life Boat Sabb Motor (p. 105) with target model 'L3 139LB' extracted exactly 6 parts strictly for Variant 2 (Y753-10001) with QTY: 2 PCS; Compressor Atlas Copco (p. 188) with target model 'LT-55' extracted exactly 20 parts strictly for LT-55/common parts (all LT22/40 parts excluded). Target Model input provision added to DB, API, ManualReview table, and Page Status modal.</t>
         </is>

</xml_diff>